<commit_message>
fix(roster): remove NG MING LIANG from 2D
He left the class. Drop him from the 2D roster, update the 2D reflection
totals (remedial /1, total /35) used when filling the RPH sheet, and add a
WITHDRAWN list so syncRoster removes him from already-saved local and
Firestore data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pupils-tracker/docs/References/namelist.xlsx
+++ b/pupils-tracker/docs/References/namelist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Claude\Pupils-tracker\pupils-tracker\docs\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DD9EA5-7945-4F24-8A7E-2C853E4C8797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29AD331C-BCCA-4437-94B2-7DBAB954F3C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>CHIN YU KAI</t>
   </si>
@@ -170,9 +170,6 @@
   </si>
   <si>
     <t>LOUIS WONG HAW TIRNG</t>
-  </si>
-  <si>
-    <t>NG MING LIANG</t>
   </si>
   <si>
     <t>ONG KAI YOU</t>
@@ -1309,13 +1306,24 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
@@ -1328,24 +1336,13 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1450,9 +1447,7 @@
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>47</v>
-      </c>
+      <c r="B11" s="1"/>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1460,7 +1455,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="2"/>
     </row>
@@ -1469,7 +1464,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="2"/>
     </row>
@@ -1478,7 +1473,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -1487,7 +1482,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2"/>
     </row>
@@ -1496,7 +1491,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="2"/>
     </row>
@@ -1505,7 +1500,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2"/>
     </row>
@@ -1514,7 +1509,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -1523,7 +1518,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C19" s="2"/>
     </row>
@@ -1532,7 +1527,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2"/>
     </row>
@@ -1541,7 +1536,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C21" s="2"/>
     </row>
@@ -1550,7 +1545,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C22" s="2"/>
     </row>
@@ -1559,7 +1554,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C23" s="2"/>
     </row>
@@ -1568,7 +1563,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C24" s="2"/>
     </row>
@@ -1577,7 +1572,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2"/>
     </row>
@@ -1586,7 +1581,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C26" s="2"/>
     </row>
@@ -1595,7 +1590,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C27" s="2"/>
     </row>
@@ -1604,7 +1599,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" s="2"/>
     </row>
@@ -1613,7 +1608,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="2"/>
     </row>
@@ -1622,7 +1617,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C30" s="2"/>
     </row>
@@ -1631,7 +1626,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C31" s="2"/>
     </row>
@@ -1640,7 +1635,7 @@
         <v>32</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C32" s="2"/>
     </row>
@@ -1649,7 +1644,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" s="2"/>
     </row>
@@ -1658,7 +1653,7 @@
         <v>34</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C34" s="2"/>
     </row>
@@ -1667,7 +1662,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C35" s="2"/>
     </row>
@@ -1676,12 +1671,36 @@
         <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -1694,30 +1713,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1733,7 +1728,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C1" s="4"/>
     </row>
@@ -1742,7 +1737,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2"/>
     </row>
@@ -1751,7 +1746,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -1760,7 +1755,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -1769,7 +1764,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -1778,7 +1773,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C6" s="2"/>
     </row>
@@ -1787,7 +1782,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -1796,7 +1791,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -1805,7 +1800,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C9" s="2"/>
     </row>
@@ -1814,7 +1809,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10" s="2"/>
     </row>
@@ -1823,7 +1818,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -1832,7 +1827,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C12" s="2"/>
     </row>
@@ -1841,7 +1836,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2"/>
     </row>
@@ -1850,7 +1845,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -1859,7 +1854,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2"/>
     </row>
@@ -1868,7 +1863,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C16" s="2"/>
     </row>
@@ -1877,7 +1872,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" s="2"/>
     </row>
@@ -1886,7 +1881,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -1895,7 +1890,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" s="2"/>
     </row>
@@ -1904,7 +1899,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C20" s="2"/>
     </row>
@@ -1913,7 +1908,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" s="2"/>
     </row>
@@ -1922,7 +1917,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C22" s="2"/>
     </row>
@@ -1931,7 +1926,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C23" s="2"/>
     </row>
@@ -1940,7 +1935,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C24" s="2"/>
     </row>
@@ -1949,7 +1944,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C25" s="2"/>
     </row>
@@ -1958,7 +1953,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C26" s="2"/>
     </row>
@@ -1967,7 +1962,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C27" s="2"/>
     </row>
@@ -1976,7 +1971,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C28" s="2"/>
     </row>
@@ -1985,7 +1980,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C29" s="2"/>
     </row>
@@ -1994,7 +1989,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C30" s="2"/>
     </row>
@@ -2003,7 +1998,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C31" s="2"/>
     </row>
@@ -2012,7 +2007,7 @@
         <v>32</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C32" s="2"/>
     </row>
@@ -2021,7 +2016,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C33" s="2"/>
     </row>
@@ -2030,7 +2025,7 @@
         <v>34</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C34" s="2"/>
     </row>
@@ -2039,7 +2034,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C35" s="2"/>
     </row>
@@ -2048,7 +2043,7 @@
         <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C36" s="2"/>
     </row>
@@ -2057,11 +2052,35 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -2074,30 +2093,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2113,7 +2108,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C1" s="4"/>
     </row>
@@ -2122,7 +2117,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2"/>
     </row>
@@ -2131,7 +2126,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -2140,7 +2135,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -2149,7 +2144,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -2158,7 +2153,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C6" s="2"/>
     </row>
@@ -2167,7 +2162,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -2176,7 +2171,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -2185,7 +2180,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2"/>
     </row>
@@ -2194,7 +2189,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2"/>
     </row>
@@ -2203,7 +2198,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -2212,7 +2207,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C12" s="2"/>
     </row>
@@ -2221,7 +2216,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C13" s="2"/>
     </row>
@@ -2230,7 +2225,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -2239,7 +2234,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C15" s="2"/>
     </row>
@@ -2248,7 +2243,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C16" s="2"/>
     </row>
@@ -2257,7 +2252,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C17" s="2"/>
     </row>
@@ -2266,7 +2261,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -2275,7 +2270,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C19" s="2"/>
     </row>
@@ -2284,7 +2279,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C20" s="2"/>
     </row>
@@ -2293,7 +2288,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C21" s="2"/>
     </row>
@@ -2302,7 +2297,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C22" s="2"/>
     </row>
@@ -2311,7 +2306,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C23" s="2"/>
     </row>
@@ -2320,7 +2315,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C24" s="2"/>
     </row>
@@ -2329,7 +2324,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C25" s="2"/>
     </row>
@@ -2338,7 +2333,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C26" s="2"/>
     </row>
@@ -2347,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C27" s="2"/>
     </row>
@@ -2356,7 +2351,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C28" s="2"/>
     </row>
@@ -2365,7 +2360,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C29" s="2"/>
     </row>
@@ -2374,7 +2369,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C30" s="2"/>
     </row>
@@ -2383,7 +2378,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C31" s="2"/>
     </row>
@@ -2392,7 +2387,7 @@
         <v>32</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C32" s="2"/>
     </row>
@@ -2401,7 +2396,7 @@
         <v>33</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C33" s="2"/>
     </row>
@@ -2410,7 +2405,7 @@
         <v>34</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C34" s="2"/>
     </row>
@@ -2419,7 +2414,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C35" s="2"/>
     </row>
@@ -2428,7 +2423,7 @@
         <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C36" s="2"/>
     </row>
@@ -2437,7 +2432,7 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -2445,33 +2440,12 @@
         <v>38</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C38" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B1:C1"/>
@@ -2488,6 +2462,27 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2503,7 +2498,7 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2511,7 +2506,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2519,7 +2514,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -2527,7 +2522,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -2535,7 +2530,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -2543,7 +2538,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -2551,7 +2546,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -2559,7 +2554,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -2567,7 +2562,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -2575,7 +2570,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -2583,7 +2578,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -2591,7 +2586,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -2599,7 +2594,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -2607,7 +2602,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -2615,7 +2610,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -2623,7 +2618,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -2631,7 +2626,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -2639,7 +2634,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -2647,7 +2642,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -2655,7 +2650,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -2663,7 +2658,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -2671,7 +2666,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -2679,7 +2674,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -2687,7 +2682,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -2695,7 +2690,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -2703,7 +2698,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -2711,7 +2706,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -2719,7 +2714,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -2727,7 +2722,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -2735,7 +2730,7 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -2743,7 +2738,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -2751,7 +2746,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -2759,7 +2754,7 @@
         <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -2767,7 +2762,7 @@
         <v>34</v>
       </c>
       <c r="B34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -2775,7 +2770,7 @@
         <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -2783,7 +2778,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -2791,7 +2786,7 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>